<commit_message>
calculate properties from FA_profile
</commit_message>
<xml_diff>
--- a/Thermodynamics/UnifacDortmund/Experimental_Data/data/acid_profile.xlsx
+++ b/Thermodynamics/UnifacDortmund/Experimental_Data/data/acid_profile.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Juan\proyectos_personales\Maestría\Materias\Tesis\oleosim\Thermodynamics\UnifacDortmund\Experimental_Data\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Juan\Maestría\Code\oleosim\Thermodynamics\UnifacDortmund\Experimental_Data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8F7A675-2C25-4CF8-BDD4-8F7270463903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2F435B-3022-4B23-811D-C7BE4350193C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -101,9 +101,6 @@
     <t>Arachidonic</t>
   </si>
   <si>
-    <t>cis-11, 14 eicosadienoic</t>
-  </si>
-  <si>
     <t>Behenic</t>
   </si>
   <si>
@@ -120,12 +117,6 @@
   </si>
   <si>
     <t>Elaidic</t>
-  </si>
-  <si>
-    <t>9,10-methylene-hexadecanoic acid</t>
-  </si>
-  <si>
-    <t>dihydrosterculic</t>
   </si>
   <si>
     <t>Paullinic</t>
@@ -161,13 +152,22 @@
     <t xml:space="preserve">No </t>
   </si>
   <si>
-    <t>Cis-9-heptadecenoic</t>
-  </si>
-  <si>
     <t>Gondoic</t>
   </si>
   <si>
     <t>Tetracosanoic</t>
+  </si>
+  <si>
+    <t>cis-9-heptadecenoic</t>
+  </si>
+  <si>
+    <t>Dihydrosterculic</t>
+  </si>
+  <si>
+    <t>cis-11,14 eicosadienoic</t>
+  </si>
+  <si>
+    <t>9,10-methylene-hexadecanoic</t>
   </si>
 </sst>
 </file>
@@ -558,36 +558,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AK126"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.26953125" customWidth="1"/>
     <col min="15" max="16" width="12" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.26953125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="12" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -628,7 +628,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>13</v>
@@ -655,66 +655,66 @@
         <v>20</v>
       </c>
       <c r="W1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="X1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AE1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AA1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AC1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AI1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AJ1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AK1" s="2" t="s">
-        <v>33</v>
-      </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F2" s="4">
         <v>0</v>
@@ -814,21 +814,21 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F3" s="4">
         <v>0</v>
@@ -924,25 +924,25 @@
         <v>0</v>
       </c>
       <c r="AK3" s="4">
-        <f>SUM(F3:AC3)</f>
+        <f t="shared" ref="AK3:AK34" si="0">SUM(F3:AC3)</f>
         <v>0.98299999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F4" s="4">
         <v>0</v>
@@ -1038,25 +1038,25 @@
         <v>0</v>
       </c>
       <c r="AK4" s="4">
-        <f>SUM(F4:AC4)</f>
+        <f t="shared" si="0"/>
         <v>1.0010000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F5" s="4">
         <v>0</v>
@@ -1152,25 +1152,25 @@
         <v>0</v>
       </c>
       <c r="AK5" s="4">
-        <f>SUM(F5:AC5)</f>
+        <f t="shared" si="0"/>
         <v>1.0009999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F6" s="4">
         <v>0</v>
@@ -1266,25 +1266,25 @@
         <v>0</v>
       </c>
       <c r="AK6" s="4">
-        <f>SUM(F6:AC6)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F7" s="4">
         <v>0</v>
@@ -1380,25 +1380,25 @@
         <v>0</v>
       </c>
       <c r="AK7" s="4">
-        <f>SUM(F7:AC7)</f>
+        <f t="shared" si="0"/>
         <v>0.98999999999999988</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F8" s="4">
         <v>0</v>
@@ -1494,25 +1494,25 @@
         <v>0</v>
       </c>
       <c r="AK8" s="4">
-        <f>SUM(F8:AC8)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F9" s="4">
         <v>0</v>
@@ -1608,25 +1608,25 @@
         <v>0</v>
       </c>
       <c r="AK9" s="4">
-        <f>SUM(F9:AC9)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F10" s="4">
         <v>0</v>
@@ -1722,25 +1722,25 @@
         <v>0</v>
       </c>
       <c r="AK10" s="4">
-        <f>SUM(F10:AC10)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F11" s="4">
         <v>0</v>
@@ -1836,25 +1836,25 @@
         <v>0</v>
       </c>
       <c r="AK11" s="4">
-        <f>SUM(F11:AC11)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F12" s="4">
         <v>0</v>
@@ -1954,25 +1954,25 @@
         <v>0</v>
       </c>
       <c r="AK12" s="4">
-        <f>SUM(F12:AC12)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>11</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F13" s="4">
         <v>2.8E-3</v>
@@ -2068,25 +2068,25 @@
         <v>0</v>
       </c>
       <c r="AK13" s="4">
-        <f>SUM(F13:AC13)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>12</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F14" s="4">
         <v>0</v>
@@ -2182,25 +2182,25 @@
         <v>0</v>
       </c>
       <c r="AK14" s="4">
-        <f>SUM(F14:AC14)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>12</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F15" s="4">
         <v>0</v>
@@ -2296,25 +2296,25 @@
         <v>0</v>
       </c>
       <c r="AK15" s="4">
-        <f>SUM(F15:AC15)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F16" s="4">
         <v>0</v>
@@ -2410,25 +2410,25 @@
         <v>0</v>
       </c>
       <c r="AK16" s="4">
-        <f>SUM(F16:AC16)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>12</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F17" s="4">
         <v>0</v>
@@ -2524,25 +2524,25 @@
         <v>0</v>
       </c>
       <c r="AK17" s="4">
-        <f>SUM(F17:AC17)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>13</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F18" s="4">
         <v>0</v>
@@ -2638,25 +2638,25 @@
         <v>0</v>
       </c>
       <c r="AK18" s="4">
-        <f>SUM(F18:AC18)</f>
+        <f t="shared" si="0"/>
         <v>0.999</v>
       </c>
     </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>14</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F19" s="4">
         <v>0</v>
@@ -2752,25 +2752,25 @@
         <v>0</v>
       </c>
       <c r="AK19" s="4">
-        <f>SUM(F19:AC19)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>15</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F20" s="4">
         <v>0</v>
@@ -2866,25 +2866,25 @@
         <v>0</v>
       </c>
       <c r="AK20" s="4">
-        <f>SUM(F20:AC20)</f>
+        <f t="shared" si="0"/>
         <v>0.99850000000000005</v>
       </c>
     </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
         <v>16</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F21" s="4">
         <v>0</v>
@@ -2980,25 +2980,25 @@
         <v>0</v>
       </c>
       <c r="AK21" s="4">
-        <f>SUM(F21:AC21)</f>
+        <f t="shared" si="0"/>
         <v>0.97</v>
       </c>
     </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>17</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F22" s="4">
         <v>0</v>
@@ -3094,25 +3094,25 @@
         <v>0</v>
       </c>
       <c r="AK22" s="4">
-        <f>SUM(F22:AC22)</f>
+        <f t="shared" si="0"/>
         <v>0.99080000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>18</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F23" s="4">
         <v>0</v>
@@ -3208,25 +3208,25 @@
         <v>0</v>
       </c>
       <c r="AK23" s="4">
-        <f>SUM(F23:AC23)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>19</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F24" s="4">
         <v>0</v>
@@ -3322,25 +3322,25 @@
         <v>0</v>
       </c>
       <c r="AK24" s="4">
-        <f>SUM(F24:AC24)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>19</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F25" s="4">
         <v>0</v>
@@ -3445,25 +3445,25 @@
         <v>0</v>
       </c>
       <c r="AK25" s="4">
-        <f>SUM(F25:AC25)</f>
+        <f t="shared" si="0"/>
         <v>0.99939999999999996</v>
       </c>
     </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
         <v>20</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F26" s="4">
         <v>0</v>
@@ -3559,25 +3559,25 @@
         <v>0</v>
       </c>
       <c r="AK26" s="4">
-        <f>SUM(F26:AC26)</f>
+        <f t="shared" si="0"/>
         <v>0.998</v>
       </c>
     </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
         <v>21</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F27" s="4">
         <v>6.0000000000000001E-3</v>
@@ -3673,25 +3673,25 @@
         <v>0</v>
       </c>
       <c r="AK27" s="4">
-        <f>SUM(F27:AC27)</f>
+        <f t="shared" si="0"/>
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A28" s="4">
         <v>22</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F28" s="4">
         <v>0</v>
@@ -3787,25 +3787,25 @@
         <v>0</v>
       </c>
       <c r="AK28" s="4">
-        <f>SUM(F28:AC28)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
         <v>23</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F29" s="4">
         <v>0</v>
@@ -3901,25 +3901,25 @@
         <v>0</v>
       </c>
       <c r="AK29" s="4">
-        <f>SUM(F29:AC29)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
         <v>23</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F30" s="4">
         <v>0</v>
@@ -4015,25 +4015,25 @@
         <v>0</v>
       </c>
       <c r="AK30" s="4">
-        <f>SUM(F30:AC30)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A31" s="4">
         <v>23</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F31" s="4">
         <v>0</v>
@@ -4129,25 +4129,25 @@
         <v>0</v>
       </c>
       <c r="AK31" s="4">
-        <f>SUM(F31:AC31)</f>
+        <f t="shared" si="0"/>
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A32" s="4">
         <v>24</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F32" s="4">
         <v>0</v>
@@ -4253,25 +4253,25 @@
         <v>0</v>
       </c>
       <c r="AK32" s="4">
-        <f>SUM(F32:AC32)</f>
+        <f t="shared" si="0"/>
         <v>0.98360000000000003</v>
       </c>
     </row>
-    <row r="33" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A33" s="4">
         <v>25</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F33" s="4">
         <v>0</v>
@@ -4375,25 +4375,25 @@
         <v>0</v>
       </c>
       <c r="AK33" s="4">
-        <f>SUM(F33:AC33)</f>
+        <f t="shared" si="0"/>
         <v>0.99089999999999989</v>
       </c>
     </row>
-    <row r="34" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A34" s="4">
         <v>26</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F34" s="4">
         <v>0</v>
@@ -4494,25 +4494,25 @@
         <v>0</v>
       </c>
       <c r="AK34" s="4">
-        <f>SUM(F34:AC34)</f>
+        <f t="shared" si="0"/>
         <v>0.996</v>
       </c>
     </row>
-    <row r="35" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A35" s="4">
         <v>26</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F35" s="4">
         <v>0</v>
@@ -4614,25 +4614,25 @@
         <v>0</v>
       </c>
       <c r="AK35" s="4">
-        <f>SUM(F35:AC35)</f>
+        <f t="shared" ref="AK35:AK66" si="1">SUM(F35:AC35)</f>
         <v>0.99769999999999992</v>
       </c>
     </row>
-    <row r="36" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A36" s="4">
         <v>27</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F36" s="4">
         <v>0</v>
@@ -4734,25 +4734,25 @@
         <v>0</v>
       </c>
       <c r="AK36" s="4">
-        <f>SUM(F36:AC36)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A37" s="4">
         <v>28</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F37" s="4">
         <v>0</v>
@@ -4857,25 +4857,25 @@
         <v>0</v>
       </c>
       <c r="AK37" s="4">
-        <f>SUM(F37:AC37)</f>
+        <f t="shared" si="1"/>
         <v>0.99132699999999996</v>
       </c>
     </row>
-    <row r="38" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A38" s="4">
         <v>29</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F38" s="5">
         <v>0</v>
@@ -4971,25 +4971,25 @@
         <v>0</v>
       </c>
       <c r="AK38" s="4">
-        <f>SUM(F38:AC38)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A39" s="4">
         <v>29</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F39" s="5">
         <v>0</v>
@@ -5085,25 +5085,25 @@
         <v>0</v>
       </c>
       <c r="AK39" s="4">
-        <f>SUM(F39:AC39)</f>
+        <f t="shared" si="1"/>
         <v>1.0001</v>
       </c>
     </row>
-    <row r="40" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A40" s="4">
         <v>29</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F40" s="5">
         <v>0</v>
@@ -5199,25 +5199,25 @@
         <v>0</v>
       </c>
       <c r="AK40" s="4">
-        <f>SUM(F40:AC40)</f>
+        <f t="shared" si="1"/>
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="41" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A41" s="4">
         <v>29</v>
       </c>
       <c r="B41" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="F41" s="5">
         <v>0</v>
@@ -5313,25 +5313,25 @@
         <v>0</v>
       </c>
       <c r="AK41" s="4">
-        <f>SUM(F41:AC41)</f>
+        <f t="shared" si="1"/>
         <v>1.0001</v>
       </c>
     </row>
-    <row r="42" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A42" s="4">
         <v>30</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F42" s="5">
         <v>0</v>
@@ -5427,25 +5427,25 @@
         <v>0</v>
       </c>
       <c r="AK42" s="4">
-        <f>SUM(F42:AC42)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A43" s="4">
         <v>30</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F43" s="5">
         <v>0</v>
@@ -5541,25 +5541,25 @@
         <v>0</v>
       </c>
       <c r="AK43" s="4">
-        <f>SUM(F43:AC43)</f>
+        <f t="shared" si="1"/>
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A44" s="4">
         <v>30</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F44" s="5">
         <v>0</v>
@@ -5655,25 +5655,25 @@
         <v>0</v>
       </c>
       <c r="AK44" s="4">
-        <f>SUM(F44:AC44)</f>
+        <f t="shared" si="1"/>
         <v>0.99880000000000013</v>
       </c>
     </row>
-    <row r="45" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A45" s="4">
         <v>30</v>
       </c>
       <c r="B45" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="F45" s="5">
         <v>0</v>
@@ -5769,25 +5769,25 @@
         <v>0</v>
       </c>
       <c r="AK45" s="4">
-        <f>SUM(F45:AC45)</f>
+        <f t="shared" si="1"/>
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A46" s="4">
         <v>31</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F46" s="5">
         <v>0</v>
@@ -5883,25 +5883,25 @@
         <v>0</v>
       </c>
       <c r="AK46" s="4">
-        <f>SUM(F46:AC46)</f>
+        <f t="shared" si="1"/>
         <v>0.99839999999999995</v>
       </c>
     </row>
-    <row r="47" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A47" s="4">
         <v>31</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F47" s="5">
         <v>0</v>
@@ -5997,25 +5997,25 @@
         <v>0</v>
       </c>
       <c r="AK47" s="4">
-        <f>SUM(F47:AC47)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A48" s="4">
         <v>32</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F48" s="5">
         <v>0</v>
@@ -6111,25 +6111,25 @@
         <v>0</v>
       </c>
       <c r="AK48" s="4">
-        <f>SUM(F48:AC48)</f>
+        <f t="shared" si="1"/>
         <v>0.996</v>
       </c>
     </row>
-    <row r="49" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A49" s="4">
         <v>32</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F49" s="5">
         <v>0</v>
@@ -6225,25 +6225,25 @@
         <v>0</v>
       </c>
       <c r="AK49" s="4">
-        <f>SUM(F49:AC49)</f>
+        <f t="shared" si="1"/>
         <v>0.996</v>
       </c>
     </row>
-    <row r="50" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A50" s="4">
         <v>33</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F50" s="5">
         <v>0</v>
@@ -6339,25 +6339,25 @@
         <v>0</v>
       </c>
       <c r="AK50" s="4">
-        <f>SUM(F50:AC50)</f>
+        <f t="shared" si="1"/>
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="51" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A51" s="4">
         <v>33</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F51" s="5">
         <v>0</v>
@@ -6453,25 +6453,25 @@
         <v>0</v>
       </c>
       <c r="AK51" s="4">
-        <f>SUM(F51:AC51)</f>
+        <f t="shared" si="1"/>
         <v>0.98050000000000004</v>
       </c>
     </row>
-    <row r="52" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A52" s="4">
         <v>34</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F52" s="5">
         <v>0</v>
@@ -6567,25 +6567,25 @@
         <v>0</v>
       </c>
       <c r="AK52" s="4">
-        <f>SUM(F52:AC52)</f>
+        <f t="shared" si="1"/>
         <v>1.0001</v>
       </c>
     </row>
-    <row r="53" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A53" s="4">
         <v>34</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F53" s="5">
         <v>0</v>
@@ -6681,25 +6681,25 @@
         <v>0</v>
       </c>
       <c r="AK53" s="4">
-        <f>SUM(F53:AC53)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A54" s="4">
         <v>34</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F54" s="5">
         <v>0</v>
@@ -6795,25 +6795,25 @@
         <v>0</v>
       </c>
       <c r="AK54" s="4">
-        <f>SUM(F54:AC54)</f>
+        <f t="shared" si="1"/>
         <v>1.0001</v>
       </c>
     </row>
-    <row r="55" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A55" s="4">
         <v>34</v>
       </c>
       <c r="B55" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E55" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E55" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="F55" s="5">
         <v>0</v>
@@ -6914,25 +6914,25 @@
         <v>0</v>
       </c>
       <c r="AK55" s="4">
-        <f>SUM(F55:AC55)</f>
+        <f t="shared" si="1"/>
         <v>0.97899999999999998</v>
       </c>
     </row>
-    <row r="56" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A56" s="4">
         <v>35</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F56" s="5">
         <v>0</v>
@@ -7028,25 +7028,25 @@
         <v>0</v>
       </c>
       <c r="AK56" s="4">
-        <f>SUM(F56:AC56)</f>
+        <f t="shared" si="1"/>
         <v>1.0001</v>
       </c>
     </row>
-    <row r="57" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A57" s="4">
         <v>35</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F57" s="5">
         <v>0</v>
@@ -7142,25 +7142,25 @@
         <v>0</v>
       </c>
       <c r="AK57" s="4">
-        <f>SUM(F57:AC57)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A58" s="4">
         <v>36</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F58" s="5">
         <v>2.5000000000000001E-3</v>
@@ -7256,25 +7256,25 @@
         <v>0</v>
       </c>
       <c r="AK58" s="4">
-        <f>SUM(F58:AC58)</f>
+        <f t="shared" si="1"/>
         <v>0.99840000000000007</v>
       </c>
     </row>
-    <row r="59" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A59" s="4">
         <v>36</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F59" s="5">
         <v>0</v>
@@ -7370,25 +7370,25 @@
         <v>0</v>
       </c>
       <c r="AK59" s="4">
-        <f>SUM(F59:AC59)</f>
+        <f t="shared" si="1"/>
         <v>0.98</v>
       </c>
     </row>
-    <row r="60" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A60" s="4">
         <v>37</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F60" s="5">
         <v>0</v>
@@ -7484,25 +7484,25 @@
         <v>0</v>
       </c>
       <c r="AK60" s="4">
-        <f>SUM(F60:AC60)</f>
+        <f t="shared" si="1"/>
         <v>0.9971000000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A61" s="4">
         <v>37</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F61" s="5">
         <v>0</v>
@@ -7598,25 +7598,25 @@
         <v>0</v>
       </c>
       <c r="AK61" s="4">
-        <f>SUM(F61:AC61)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A62" s="4">
         <v>37</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F62" s="5">
         <v>0</v>
@@ -7712,25 +7712,25 @@
         <v>0</v>
       </c>
       <c r="AK62" s="4">
-        <f>SUM(F62:AC62)</f>
+        <f t="shared" si="1"/>
         <v>0.99920000000000009</v>
       </c>
     </row>
-    <row r="63" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A63" s="4">
         <v>37</v>
       </c>
       <c r="B63" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E63" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E63" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="F63" s="5">
         <v>0</v>
@@ -7826,25 +7826,25 @@
         <v>0</v>
       </c>
       <c r="AK63" s="4">
-        <f>SUM(F63:AC63)</f>
+        <f t="shared" si="1"/>
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="64" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A64" s="4">
         <v>37</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F64" s="5">
         <v>0</v>
@@ -7940,25 +7940,25 @@
         <v>0</v>
       </c>
       <c r="AK64" s="4">
-        <f>SUM(F64:AC64)</f>
+        <f t="shared" si="1"/>
         <v>0.99670000000000003</v>
       </c>
     </row>
-    <row r="65" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A65" s="4">
         <v>37</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F65" s="5">
         <v>0</v>
@@ -8054,25 +8054,25 @@
         <v>0</v>
       </c>
       <c r="AK65" s="4">
-        <f>SUM(F65:AC65)</f>
+        <f t="shared" si="1"/>
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="66" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A66" s="4">
         <v>38</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F66" s="5">
         <v>0</v>
@@ -8168,25 +8168,25 @@
         <v>0</v>
       </c>
       <c r="AK66" s="4">
-        <f>SUM(F66:AC66)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A67" s="4">
         <v>38</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F67" s="5">
         <v>0</v>
@@ -8282,25 +8282,25 @@
         <v>0</v>
       </c>
       <c r="AK67" s="4">
-        <f>SUM(F67:AC67)</f>
+        <f t="shared" ref="AK67:AK98" si="2">SUM(F67:AC67)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A68" s="4">
         <v>39</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F68" s="5">
         <v>0</v>
@@ -8396,25 +8396,25 @@
         <v>0</v>
       </c>
       <c r="AK68" s="4">
-        <f>SUM(F68:AC68)</f>
+        <f t="shared" si="2"/>
         <v>0.995</v>
       </c>
     </row>
-    <row r="69" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A69" s="4">
         <v>39</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F69" s="5">
         <v>0</v>
@@ -8510,25 +8510,25 @@
         <v>0</v>
       </c>
       <c r="AK69" s="4">
-        <f>SUM(F69:AC69)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A70" s="4">
         <v>39</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F70" s="5">
         <v>0</v>
@@ -8624,25 +8624,25 @@
         <v>0</v>
       </c>
       <c r="AK70" s="4">
-        <f>SUM(F70:AC70)</f>
+        <f t="shared" si="2"/>
         <v>0.9920000000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A71" s="4">
         <v>39</v>
       </c>
       <c r="B71" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E71" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="F71" s="5">
         <v>0</v>
@@ -8738,25 +8738,25 @@
         <v>0</v>
       </c>
       <c r="AK71" s="4">
-        <f>SUM(F71:AC71)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A72" s="4">
         <v>40</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F72" s="5">
         <v>0</v>
@@ -8852,25 +8852,25 @@
         <v>0</v>
       </c>
       <c r="AK72" s="4">
-        <f>SUM(F72:AC72)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A73" s="4">
         <v>40</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F73" s="5">
         <v>0</v>
@@ -8966,25 +8966,25 @@
         <v>0</v>
       </c>
       <c r="AK73" s="4">
-        <f>SUM(F73:AC73)</f>
+        <f t="shared" si="2"/>
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="74" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A74" s="4">
         <v>41</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F74" s="5">
         <v>0</v>
@@ -9080,25 +9080,25 @@
         <v>0</v>
       </c>
       <c r="AK74" s="4">
-        <f>SUM(F74:AC74)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A75" s="4">
         <v>41</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F75" s="5">
         <v>0</v>
@@ -9194,25 +9194,25 @@
         <v>0</v>
       </c>
       <c r="AK75" s="4">
-        <f>SUM(F75:AC75)</f>
+        <f t="shared" si="2"/>
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A76" s="4">
         <v>42</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F76" s="5">
         <v>0</v>
@@ -9308,25 +9308,25 @@
         <v>0</v>
       </c>
       <c r="AK76" s="4">
-        <f>SUM(F76:AC76)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A77" s="4">
         <v>42</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F77" s="5">
         <v>0</v>
@@ -9422,25 +9422,25 @@
         <v>0</v>
       </c>
       <c r="AK77" s="4">
-        <f>SUM(F77:AC77)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A78" s="4">
         <v>42</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F78" s="5">
         <v>0</v>
@@ -9536,25 +9536,25 @@
         <v>0</v>
       </c>
       <c r="AK78" s="4">
-        <f>SUM(F78:AC78)</f>
+        <f t="shared" si="2"/>
         <v>0.97529999999999994</v>
       </c>
     </row>
-    <row r="79" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A79" s="4">
         <v>42</v>
       </c>
       <c r="B79" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E79" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="F79" s="5">
         <v>0</v>
@@ -9650,25 +9650,25 @@
         <v>0</v>
       </c>
       <c r="AK79" s="4">
-        <f>SUM(F79:AC79)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A80" s="4">
         <v>43</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F80" s="5">
         <v>0</v>
@@ -9764,25 +9764,25 @@
         <v>0</v>
       </c>
       <c r="AK80" s="4">
-        <f>SUM(F80:AC80)</f>
+        <f t="shared" si="2"/>
         <v>0.99770000000000003</v>
       </c>
     </row>
-    <row r="81" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A81" s="4">
         <v>43</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F81" s="5">
         <v>0</v>
@@ -9878,25 +9878,25 @@
         <v>0</v>
       </c>
       <c r="AK81" s="4">
-        <f>SUM(F81:AC81)</f>
+        <f t="shared" si="2"/>
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="82" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A82" s="4">
         <v>44</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F82" s="5">
         <v>0</v>
@@ -9992,25 +9992,25 @@
         <v>0</v>
       </c>
       <c r="AK82" s="4">
-        <f>SUM(F82:AC82)</f>
+        <f t="shared" si="2"/>
         <v>0.9988999999999999</v>
       </c>
     </row>
-    <row r="83" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A83" s="4">
         <v>44</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F83" s="5">
         <v>1E-3</v>
@@ -10112,25 +10112,25 @@
         <v>0</v>
       </c>
       <c r="AK83" s="4">
-        <f>SUM(F83:AC83)</f>
+        <f t="shared" si="2"/>
         <v>0.93859999999999988</v>
       </c>
     </row>
-    <row r="84" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A84" s="4">
         <v>44</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F84" s="5">
         <v>0</v>
@@ -10230,25 +10230,25 @@
         <v>0</v>
       </c>
       <c r="AK84" s="4">
-        <f>SUM(F84:AC84)</f>
+        <f t="shared" si="2"/>
         <v>0.99809999999999999</v>
       </c>
     </row>
-    <row r="85" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A85" s="4">
         <v>44</v>
       </c>
       <c r="B85" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E85" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="F85" s="5">
         <v>1E-3</v>
@@ -10350,25 +10350,25 @@
         <v>0</v>
       </c>
       <c r="AK85" s="4">
-        <f>SUM(F85:AC85)</f>
+        <f t="shared" si="2"/>
         <v>0.93859999999999988</v>
       </c>
     </row>
-    <row r="86" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A86" s="4">
         <v>45</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F86" s="5">
         <v>0</v>
@@ -10464,25 +10464,25 @@
         <v>0</v>
       </c>
       <c r="AK86" s="4">
-        <f>SUM(F86:AC86)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A87" s="4">
         <v>45</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F87" s="5">
         <v>0</v>
@@ -10578,25 +10578,25 @@
         <v>0</v>
       </c>
       <c r="AK87" s="4">
-        <f>SUM(F87:AC87)</f>
+        <f t="shared" si="2"/>
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="88" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A88" s="4">
         <v>46</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F88" s="5">
         <v>0.10580000000000001</v>
@@ -10692,25 +10692,25 @@
         <v>0</v>
       </c>
       <c r="AK88" s="4">
-        <f>SUM(F88:AC88)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A89" s="4">
         <v>46</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F89" s="5">
         <v>0</v>
@@ -10806,25 +10806,25 @@
         <v>0</v>
       </c>
       <c r="AK89" s="4">
-        <f>SUM(F89:AC89)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A90" s="4">
         <v>47</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F90" s="5">
         <v>0</v>
@@ -10920,25 +10920,25 @@
         <v>0</v>
       </c>
       <c r="AK90" s="4">
-        <f>SUM(F90:AC90)</f>
+        <f t="shared" si="2"/>
         <v>1.0001</v>
       </c>
     </row>
-    <row r="91" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A91" s="4">
         <v>47</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F91" s="5">
         <v>0</v>
@@ -11034,25 +11034,25 @@
         <v>0</v>
       </c>
       <c r="AK91" s="4">
-        <f>SUM(F91:AC91)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A92" s="4">
         <v>47</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F92" s="5">
         <v>0</v>
@@ -11148,25 +11148,25 @@
         <v>0</v>
       </c>
       <c r="AK92" s="4">
-        <f>SUM(F92:AC92)</f>
+        <f t="shared" si="2"/>
         <v>1.0001</v>
       </c>
     </row>
-    <row r="93" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A93" s="4">
         <v>48</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F93" s="4">
         <v>0</v>
@@ -11262,25 +11262,25 @@
         <v>0</v>
       </c>
       <c r="AK93" s="4">
-        <f>SUM(F93:AC93)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A94" s="4">
         <v>48</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F94" s="4">
         <v>0</v>
@@ -11376,25 +11376,25 @@
         <v>0</v>
       </c>
       <c r="AK94" s="4">
-        <f>SUM(F94:AC94)</f>
+        <f t="shared" si="2"/>
         <v>0.99080000000000001</v>
       </c>
     </row>
-    <row r="95" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A95" s="4">
         <v>49</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F95" s="5">
         <v>0</v>
@@ -11499,25 +11499,25 @@
         <v>0</v>
       </c>
       <c r="AK95" s="4">
-        <f>SUM(F95:AC95)</f>
+        <f t="shared" si="2"/>
         <v>0.99030000000000018</v>
       </c>
     </row>
-    <row r="96" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A96" s="4">
         <v>49</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F96" s="5">
         <v>0</v>
@@ -11613,25 +11613,25 @@
         <v>0</v>
       </c>
       <c r="AK96" s="4">
-        <f>SUM(F96:AC96)</f>
+        <f t="shared" si="2"/>
         <v>0.99600000000000011</v>
       </c>
     </row>
-    <row r="97" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A97" s="4">
         <v>49</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F97" s="5">
         <v>0</v>
@@ -11727,25 +11727,25 @@
         <v>0</v>
       </c>
       <c r="AK97" s="4">
-        <f>SUM(F97:AC97)</f>
+        <f t="shared" si="2"/>
         <v>0.99550000000000005</v>
       </c>
     </row>
-    <row r="98" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A98" s="4">
         <v>49</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F98" s="5">
         <v>0</v>
@@ -11841,25 +11841,25 @@
         <v>0</v>
       </c>
       <c r="AK98" s="4">
-        <f>SUM(F98:AC98)</f>
+        <f t="shared" si="2"/>
         <v>0.99730000000000008</v>
       </c>
     </row>
-    <row r="99" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A99" s="4">
         <v>49</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F99" s="5">
         <v>0</v>
@@ -11955,25 +11955,25 @@
         <v>0</v>
       </c>
       <c r="AK99" s="4">
-        <f>SUM(F99:AC99)</f>
+        <f t="shared" ref="AK99:AK112" si="3">SUM(F99:AC99)</f>
         <v>0.99709999999999988</v>
       </c>
     </row>
-    <row r="100" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A100" s="4">
         <v>49</v>
       </c>
       <c r="B100" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C100" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C100" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="D100" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F100" s="5">
         <v>0</v>
@@ -12069,25 +12069,25 @@
         <v>0</v>
       </c>
       <c r="AK100" s="4">
-        <f>SUM(F100:AC100)</f>
+        <f t="shared" si="3"/>
         <v>0.99600000000000011</v>
       </c>
     </row>
-    <row r="101" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A101" s="4">
         <v>49</v>
       </c>
       <c r="B101" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D101" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C101" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D101" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="E101" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F101" s="5">
         <v>0</v>
@@ -12183,25 +12183,25 @@
         <v>0</v>
       </c>
       <c r="AK101" s="4">
-        <f>SUM(F101:AC101)</f>
+        <f t="shared" si="3"/>
         <v>0.99550000000000005</v>
       </c>
     </row>
-    <row r="102" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A102" s="4">
         <v>49</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F102" s="5">
         <v>0</v>
@@ -12297,25 +12297,25 @@
         <v>0</v>
       </c>
       <c r="AK102" s="4">
-        <f>SUM(F102:AC102)</f>
+        <f t="shared" si="3"/>
         <v>0.99730000000000008</v>
       </c>
     </row>
-    <row r="103" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A103" s="4">
         <v>49</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F103" s="5">
         <v>0</v>
@@ -12411,25 +12411,25 @@
         <v>0</v>
       </c>
       <c r="AK103" s="4">
-        <f>SUM(F103:AC103)</f>
+        <f t="shared" si="3"/>
         <v>0.98720000000000008</v>
       </c>
     </row>
-    <row r="104" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A104" s="4">
         <v>49</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F104" s="5">
         <v>0</v>
@@ -12525,25 +12525,25 @@
         <v>0</v>
       </c>
       <c r="AK104" s="4">
-        <f>SUM(F104:AC104)</f>
+        <f t="shared" si="3"/>
         <v>0.99600000000000011</v>
       </c>
     </row>
-    <row r="105" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A105" s="4">
         <v>49</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F105" s="5">
         <v>0</v>
@@ -12639,25 +12639,25 @@
         <v>0</v>
       </c>
       <c r="AK105" s="4">
-        <f>SUM(F105:AC105)</f>
+        <f t="shared" si="3"/>
         <v>0.99419999999999986</v>
       </c>
     </row>
-    <row r="106" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A106" s="4">
         <v>49</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F106" s="5">
         <v>0</v>
@@ -12753,25 +12753,25 @@
         <v>0</v>
       </c>
       <c r="AK106" s="4">
-        <f>SUM(F106:AC106)</f>
+        <f t="shared" si="3"/>
         <v>0.99770000000000003</v>
       </c>
     </row>
-    <row r="107" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A107" s="4">
         <v>50</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F107" s="5">
         <v>0</v>
@@ -12874,25 +12874,25 @@
         <v>0</v>
       </c>
       <c r="AK107" s="4">
-        <f>SUM(F107:AC107)</f>
+        <f t="shared" si="3"/>
         <v>0.99580000000000002</v>
       </c>
     </row>
-    <row r="108" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A108" s="4">
         <v>50</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F108" s="5">
         <v>0</v>
@@ -12988,25 +12988,25 @@
         <v>0</v>
       </c>
       <c r="AK108" s="4">
-        <f>SUM(F108:AC108)</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A109" s="4">
         <v>50</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F109" s="5">
         <v>0</v>
@@ -13108,25 +13108,25 @@
         <v>0</v>
       </c>
       <c r="AK109" s="4">
-        <f>SUM(F109:AC109)</f>
+        <f t="shared" si="3"/>
         <v>0.998</v>
       </c>
     </row>
-    <row r="110" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A110" s="4">
         <v>50</v>
       </c>
       <c r="B110" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C110" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C110" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="D110" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F110" s="5">
         <v>0</v>
@@ -13222,25 +13222,25 @@
         <v>0</v>
       </c>
       <c r="AK110" s="4">
-        <f>SUM(F110:AC110)</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A111" s="4">
         <v>50</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F111" s="5">
         <v>0</v>
@@ -13344,25 +13344,25 @@
         <v>0</v>
       </c>
       <c r="AK111" s="4">
-        <f>SUM(F111:AC111)</f>
+        <f t="shared" si="3"/>
         <v>1.0010000000000001</v>
       </c>
     </row>
-    <row r="112" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A112" s="4">
         <v>50</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F112" s="5">
         <v>0</v>
@@ -13458,25 +13458,25 @@
         <v>0</v>
       </c>
       <c r="AK112" s="4">
-        <f>SUM(F112:AC112)</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A113" s="4">
         <v>51</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F113" s="5">
         <v>0</v>
@@ -13585,21 +13585,21 @@
         <v>0.9900000000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A114" s="4">
         <v>52</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F114" s="5">
         <v>0</v>
@@ -13704,21 +13704,21 @@
         <v>0.99902599999999997</v>
       </c>
     </row>
-    <row r="115" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A115" s="4">
         <v>53</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F115" s="5">
         <v>0</v>
@@ -13822,21 +13822,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A116" s="4">
         <v>54</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F116" s="5">
         <v>0</v>
@@ -13936,21 +13936,21 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="117" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A117" s="4">
         <v>55</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F117" s="4">
         <v>0</v>
@@ -14046,25 +14046,25 @@
         <v>0</v>
       </c>
       <c r="AK117" s="4">
-        <f t="shared" ref="AK117:AK126" si="0">SUM(F117:AJ117)</f>
+        <f t="shared" ref="AK117:AK126" si="4">SUM(F117:AJ117)</f>
         <v>0.99990000000000012</v>
       </c>
     </row>
-    <row r="118" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A118" s="4">
         <v>55</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F118" s="4">
         <v>0</v>
@@ -14160,25 +14160,25 @@
         <v>0</v>
       </c>
       <c r="AK118" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0.99829999999999997</v>
       </c>
     </row>
-    <row r="119" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A119" s="4">
         <v>55</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F119" s="4">
         <v>0</v>
@@ -14274,25 +14274,25 @@
         <v>0</v>
       </c>
       <c r="AK119" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>1.0000999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A120" s="4">
         <v>55</v>
       </c>
       <c r="B120" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C120" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C120" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="D120" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F120" s="4">
         <v>0</v>
@@ -14388,25 +14388,25 @@
         <v>0</v>
       </c>
       <c r="AK120" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0.99829999999999997</v>
       </c>
     </row>
-    <row r="121" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A121" s="4">
         <v>55</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F121" s="4">
         <v>0</v>
@@ -14502,25 +14502,25 @@
         <v>0</v>
       </c>
       <c r="AK121" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>1.0002000000000002</v>
       </c>
     </row>
-    <row r="122" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A122" s="4">
         <v>55</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F122" s="4">
         <v>0</v>
@@ -14616,25 +14616,25 @@
         <v>0</v>
       </c>
       <c r="AK122" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0.99829999999999997</v>
       </c>
     </row>
-    <row r="123" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A123" s="4">
         <v>56</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F123" s="4">
         <v>0</v>
@@ -14730,25 +14730,25 @@
         <v>0</v>
       </c>
       <c r="AK123" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0.98139999999999994</v>
       </c>
     </row>
-    <row r="124" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A124" s="4">
         <v>56</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F124" s="4">
         <v>0</v>
@@ -14844,25 +14844,25 @@
         <v>0</v>
       </c>
       <c r="AK124" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0.98007600000000017</v>
       </c>
     </row>
-    <row r="125" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A125" s="4">
         <v>56</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F125" s="4">
         <v>0</v>
@@ -14958,25 +14958,25 @@
         <v>0</v>
       </c>
       <c r="AK125" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0.97875199999999996</v>
       </c>
     </row>
-    <row r="126" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A126" s="4">
         <v>57</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F126" s="4">
         <v>0</v>
@@ -15072,7 +15072,7 @@
         <v>0</v>
       </c>
       <c r="AK126" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated m, n, p coefficient calculation
</commit_message>
<xml_diff>
--- a/Thermodynamics/UnifacDortmund/Experimental_Data/data/acid_profile.xlsx
+++ b/Thermodynamics/UnifacDortmund/Experimental_Data/data/acid_profile.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Juan\Maestría\Code\oleosim\Thermodynamics\UnifacDortmund\Experimental_Data\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Juan\proyectos_personales\Maestría\Materias\Tesis\oleosim\Thermodynamics\UnifacDortmund\Experimental_Data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2F435B-3022-4B23-811D-C7BE4350193C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8536949A-305A-49B9-B631-1F43AA9DC789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -558,36 +558,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AK126"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.26953125" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.28515625" customWidth="1"/>
     <col min="15" max="16" width="12" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="12" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.81640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="32.453125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -700,7 +700,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -814,7 +814,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -928,7 +928,7 @@
         <v>0.98299999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>1.0010000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>1.0009999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1270,7 +1270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>0.98999999999999988</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1612,7 +1612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>11</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>12</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>12</v>
       </c>
@@ -2300,7 +2300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>12</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>12</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>13</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>14</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>15</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>0.99850000000000005</v>
       </c>
     </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>16</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>17</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>0.99080000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>18</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>19</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>19</v>
       </c>
@@ -3449,7 +3449,7 @@
         <v>0.99939999999999996</v>
       </c>
     </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>20</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>21</v>
       </c>
@@ -3677,7 +3677,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>22</v>
       </c>
@@ -3791,7 +3791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>23</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>23</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>23</v>
       </c>
@@ -4133,7 +4133,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>24</v>
       </c>
@@ -4161,7 +4161,9 @@
       <c r="I32" s="4">
         <v>0</v>
       </c>
-      <c r="J32" s="4"/>
+      <c r="J32" s="4">
+        <v>0</v>
+      </c>
       <c r="K32" s="4">
         <f>4.04/100</f>
         <v>4.0399999999999998E-2</v>
@@ -4257,7 +4259,7 @@
         <v>0.98360000000000003</v>
       </c>
     </row>
-    <row r="33" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>25</v>
       </c>
@@ -4379,7 +4381,7 @@
         <v>0.99089999999999989</v>
       </c>
     </row>
-    <row r="34" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>26</v>
       </c>
@@ -4498,7 +4500,7 @@
         <v>0.996</v>
       </c>
     </row>
-    <row r="35" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>26</v>
       </c>
@@ -4618,7 +4620,7 @@
         <v>0.99769999999999992</v>
       </c>
     </row>
-    <row r="36" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>27</v>
       </c>
@@ -4738,7 +4740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>28</v>
       </c>
@@ -4861,7 +4863,7 @@
         <v>0.99132699999999996</v>
       </c>
     </row>
-    <row r="38" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
         <v>29</v>
       </c>
@@ -4975,7 +4977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
         <v>29</v>
       </c>
@@ -5089,7 +5091,7 @@
         <v>1.0001</v>
       </c>
     </row>
-    <row r="40" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>29</v>
       </c>
@@ -5203,7 +5205,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="41" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>29</v>
       </c>
@@ -5317,7 +5319,7 @@
         <v>1.0001</v>
       </c>
     </row>
-    <row r="42" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>30</v>
       </c>
@@ -5431,7 +5433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>30</v>
       </c>
@@ -5545,7 +5547,7 @@
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
         <v>30</v>
       </c>
@@ -5659,7 +5661,7 @@
         <v>0.99880000000000013</v>
       </c>
     </row>
-    <row r="45" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>30</v>
       </c>
@@ -5773,7 +5775,7 @@
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>31</v>
       </c>
@@ -5887,7 +5889,7 @@
         <v>0.99839999999999995</v>
       </c>
     </row>
-    <row r="47" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>31</v>
       </c>
@@ -6001,7 +6003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>32</v>
       </c>
@@ -6115,7 +6117,7 @@
         <v>0.996</v>
       </c>
     </row>
-    <row r="49" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>32</v>
       </c>
@@ -6229,7 +6231,7 @@
         <v>0.996</v>
       </c>
     </row>
-    <row r="50" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
         <v>33</v>
       </c>
@@ -6343,7 +6345,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="51" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>33</v>
       </c>
@@ -6457,7 +6459,7 @@
         <v>0.98050000000000004</v>
       </c>
     </row>
-    <row r="52" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>34</v>
       </c>
@@ -6571,7 +6573,7 @@
         <v>1.0001</v>
       </c>
     </row>
-    <row r="53" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>34</v>
       </c>
@@ -6685,7 +6687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>34</v>
       </c>
@@ -6799,7 +6801,7 @@
         <v>1.0001</v>
       </c>
     </row>
-    <row r="55" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>34</v>
       </c>
@@ -6918,7 +6920,7 @@
         <v>0.97899999999999998</v>
       </c>
     </row>
-    <row r="56" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>35</v>
       </c>
@@ -7032,7 +7034,7 @@
         <v>1.0001</v>
       </c>
     </row>
-    <row r="57" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>35</v>
       </c>
@@ -7146,7 +7148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>36</v>
       </c>
@@ -7260,7 +7262,7 @@
         <v>0.99840000000000007</v>
       </c>
     </row>
-    <row r="59" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
         <v>36</v>
       </c>
@@ -7374,7 +7376,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="60" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
         <v>37</v>
       </c>
@@ -7488,7 +7490,7 @@
         <v>0.9971000000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>37</v>
       </c>
@@ -7602,7 +7604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
         <v>37</v>
       </c>
@@ -7716,7 +7718,7 @@
         <v>0.99920000000000009</v>
       </c>
     </row>
-    <row r="63" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>37</v>
       </c>
@@ -7830,7 +7832,7 @@
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="64" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>37</v>
       </c>
@@ -7944,7 +7946,7 @@
         <v>0.99670000000000003</v>
       </c>
     </row>
-    <row r="65" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>37</v>
       </c>
@@ -8058,7 +8060,7 @@
         <v>0.99990000000000001</v>
       </c>
     </row>
-    <row r="66" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>38</v>
       </c>
@@ -8172,7 +8174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>38</v>
       </c>
@@ -8286,7 +8288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>39</v>
       </c>
@@ -8400,7 +8402,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="69" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>39</v>
       </c>
@@ -8514,7 +8516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>39</v>
       </c>
@@ -8628,7 +8630,7 @@
         <v>0.9920000000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>39</v>
       </c>
@@ -8742,7 +8744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>40</v>
       </c>
@@ -8856,7 +8858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>40</v>
       </c>
@@ -8970,7 +8972,7 @@
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="74" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>41</v>
       </c>
@@ -9084,7 +9086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>41</v>
       </c>
@@ -9198,7 +9200,7 @@
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>42</v>
       </c>
@@ -9312,7 +9314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>42</v>
       </c>
@@ -9426,7 +9428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>42</v>
       </c>
@@ -9540,7 +9542,7 @@
         <v>0.97529999999999994</v>
       </c>
     </row>
-    <row r="79" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>42</v>
       </c>
@@ -9654,7 +9656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>43</v>
       </c>
@@ -9768,7 +9770,7 @@
         <v>0.99770000000000003</v>
       </c>
     </row>
-    <row r="81" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>43</v>
       </c>
@@ -9882,7 +9884,7 @@
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="82" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>44</v>
       </c>
@@ -9996,7 +9998,7 @@
         <v>0.9988999999999999</v>
       </c>
     </row>
-    <row r="83" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>44</v>
       </c>
@@ -10116,7 +10118,7 @@
         <v>0.93859999999999988</v>
       </c>
     </row>
-    <row r="84" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>44</v>
       </c>
@@ -10234,7 +10236,7 @@
         <v>0.99809999999999999</v>
       </c>
     </row>
-    <row r="85" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>44</v>
       </c>
@@ -10354,7 +10356,7 @@
         <v>0.93859999999999988</v>
       </c>
     </row>
-    <row r="86" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
         <v>45</v>
       </c>
@@ -10468,7 +10470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
         <v>45</v>
       </c>
@@ -10582,7 +10584,7 @@
         <v>0.98080000000000001</v>
       </c>
     </row>
-    <row r="88" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
         <v>46</v>
       </c>
@@ -10696,7 +10698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
         <v>46</v>
       </c>
@@ -10810,7 +10812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
         <v>47</v>
       </c>
@@ -10924,7 +10926,7 @@
         <v>1.0001</v>
       </c>
     </row>
-    <row r="91" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
         <v>47</v>
       </c>
@@ -11038,7 +11040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
         <v>47</v>
       </c>
@@ -11152,7 +11154,7 @@
         <v>1.0001</v>
       </c>
     </row>
-    <row r="93" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
         <v>48</v>
       </c>
@@ -11266,7 +11268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
         <v>48</v>
       </c>
@@ -11380,7 +11382,7 @@
         <v>0.99080000000000001</v>
       </c>
     </row>
-    <row r="95" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
         <v>49</v>
       </c>
@@ -11503,7 +11505,7 @@
         <v>0.99030000000000018</v>
       </c>
     </row>
-    <row r="96" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
         <v>49</v>
       </c>
@@ -11617,7 +11619,7 @@
         <v>0.99600000000000011</v>
       </c>
     </row>
-    <row r="97" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
         <v>49</v>
       </c>
@@ -11731,7 +11733,7 @@
         <v>0.99550000000000005</v>
       </c>
     </row>
-    <row r="98" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
         <v>49</v>
       </c>
@@ -11845,7 +11847,7 @@
         <v>0.99730000000000008</v>
       </c>
     </row>
-    <row r="99" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
         <v>49</v>
       </c>
@@ -11959,7 +11961,7 @@
         <v>0.99709999999999988</v>
       </c>
     </row>
-    <row r="100" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>49</v>
       </c>
@@ -12073,7 +12075,7 @@
         <v>0.99600000000000011</v>
       </c>
     </row>
-    <row r="101" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>49</v>
       </c>
@@ -12187,7 +12189,7 @@
         <v>0.99550000000000005</v>
       </c>
     </row>
-    <row r="102" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
         <v>49</v>
       </c>
@@ -12301,7 +12303,7 @@
         <v>0.99730000000000008</v>
       </c>
     </row>
-    <row r="103" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
         <v>49</v>
       </c>
@@ -12415,7 +12417,7 @@
         <v>0.98720000000000008</v>
       </c>
     </row>
-    <row r="104" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
         <v>49</v>
       </c>
@@ -12529,7 +12531,7 @@
         <v>0.99600000000000011</v>
       </c>
     </row>
-    <row r="105" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
         <v>49</v>
       </c>
@@ -12643,7 +12645,7 @@
         <v>0.99419999999999986</v>
       </c>
     </row>
-    <row r="106" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
         <v>49</v>
       </c>
@@ -12757,7 +12759,7 @@
         <v>0.99770000000000003</v>
       </c>
     </row>
-    <row r="107" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
         <v>50</v>
       </c>
@@ -12878,7 +12880,7 @@
         <v>0.99580000000000002</v>
       </c>
     </row>
-    <row r="108" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
         <v>50</v>
       </c>
@@ -12992,7 +12994,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
         <v>50</v>
       </c>
@@ -13112,7 +13114,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="110" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>50</v>
       </c>
@@ -13226,7 +13228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
         <v>50</v>
       </c>
@@ -13348,7 +13350,7 @@
         <v>1.0010000000000001</v>
       </c>
     </row>
-    <row r="112" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
         <v>50</v>
       </c>
@@ -13462,7 +13464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
         <v>51</v>
       </c>
@@ -13585,7 +13587,7 @@
         <v>0.9900000000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
         <v>52</v>
       </c>
@@ -13704,7 +13706,7 @@
         <v>0.99902599999999997</v>
       </c>
     </row>
-    <row r="115" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
         <v>53</v>
       </c>
@@ -13822,7 +13824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
         <v>54</v>
       </c>
@@ -13936,7 +13938,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="117" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
         <v>55</v>
       </c>
@@ -14050,7 +14052,7 @@
         <v>0.99990000000000012</v>
       </c>
     </row>
-    <row r="118" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
         <v>55</v>
       </c>
@@ -14164,7 +14166,7 @@
         <v>0.99829999999999997</v>
       </c>
     </row>
-    <row r="119" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
         <v>55</v>
       </c>
@@ -14278,7 +14280,7 @@
         <v>1.0000999999999998</v>
       </c>
     </row>
-    <row r="120" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
         <v>55</v>
       </c>
@@ -14392,7 +14394,7 @@
         <v>0.99829999999999997</v>
       </c>
     </row>
-    <row r="121" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
         <v>55</v>
       </c>
@@ -14506,7 +14508,7 @@
         <v>1.0002000000000002</v>
       </c>
     </row>
-    <row r="122" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
         <v>55</v>
       </c>
@@ -14620,7 +14622,7 @@
         <v>0.99829999999999997</v>
       </c>
     </row>
-    <row r="123" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
         <v>56</v>
       </c>
@@ -14734,7 +14736,7 @@
         <v>0.98139999999999994</v>
       </c>
     </row>
-    <row r="124" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
         <v>56</v>
       </c>
@@ -14848,7 +14850,7 @@
         <v>0.98007600000000017</v>
       </c>
     </row>
-    <row r="125" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
         <v>56</v>
       </c>
@@ -14962,7 +14964,7 @@
         <v>0.97875199999999996</v>
       </c>
     </row>
-    <row r="126" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
         <v>57</v>
       </c>

</xml_diff>